<commit_message>
CSV support, per-column date parsing, trend charts, clearer structure, write-up
- Accept .csv and .xls as well as .xlsx; a CSV is loaded as one sheet and cleaned the same way
- Decide day-first vs month-first once per date column (01/08 was being read as 8 January)
- Reject joins whose columns share no values, so an invented link gives a refusal, not zeros
- Rank target comparisons by percentage and return the top 5 for "which is highest" questions
- Charts: one line per category for trends split by a group, value labels, no hover toolbar
- Rewrite the answer sentence when it misquotes a number from the result
- Rename core/ to excel_qa/ with one job per module; shorter comments; prompts in one file
- Sample data: three linked workbooks plus a returns CSV; README and one-page write-up

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/customers.xlsx
+++ b/samples/customers.xlsx
@@ -456,17 +456,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Customer 0</t>
+          <t>Greenharbor Retail</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>SMB</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>South</t>
         </is>
       </c>
       <c r="E2" s="1" t="n">
@@ -481,7 +481,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Customer 1</t>
+          <t>Silverstone Foods</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -506,17 +506,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Customer 2</t>
+          <t>Greenworks Systems</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Enterprise</t>
+          <t>SMB</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>West</t>
         </is>
       </c>
       <c r="E4" s="1" t="n">
@@ -531,17 +531,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Customer 3</t>
+          <t>Mapleriver Traders</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Enterprise</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>South</t>
         </is>
       </c>
       <c r="E5" s="1" t="n">
@@ -556,17 +556,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Customer 4</t>
+          <t>Bluefield Logistics</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>SMB</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>East</t>
         </is>
       </c>
       <c r="E6" s="1" t="n">
@@ -581,17 +581,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Customer 5</t>
+          <t>Silverworks Traders</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Enterprise</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>West</t>
         </is>
       </c>
       <c r="E7" s="1" t="n">
@@ -606,17 +606,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Customer 6</t>
+          <t>Summitstone Textiles</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Enterprise</t>
+          <t>SMB</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>South</t>
         </is>
       </c>
       <c r="E8" s="1" t="n">
@@ -631,17 +631,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Customer 7</t>
+          <t>Silvergate Retail</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Enterprise</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>South</t>
         </is>
       </c>
       <c r="E9" s="1" t="n">
@@ -656,12 +656,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Customer 8</t>
+          <t>Bluebridge Textiles</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Enterprise</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -681,17 +681,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Customer 9</t>
+          <t>Urbanleaf Foods</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Enterprise</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>West</t>
         </is>
       </c>
       <c r="E11" s="1" t="n">
@@ -706,12 +706,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Customer 10</t>
+          <t>Silverpeak Systems</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Enterprise</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Customer 11</t>
+          <t>Greenriver Systems</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -741,7 +741,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>West</t>
         </is>
       </c>
       <c r="E13" s="1" t="n">
@@ -756,12 +756,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Customer 12</t>
+          <t>Urbanpeak Retail</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>SMB</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -781,12 +781,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Customer 13</t>
+          <t>Bluegate Systems</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enterprise</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Customer 14</t>
+          <t>Primefield Retail</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>South</t>
         </is>
       </c>
       <c r="E16" s="1" t="n">
@@ -831,17 +831,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Customer 15</t>
+          <t>Maplepeak Logistics</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>SMB</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>South</t>
         </is>
       </c>
       <c r="E17" s="1" t="n">
@@ -856,7 +856,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Customer 16</t>
+          <t>Greenharbor Logistics</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -866,7 +866,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>North</t>
         </is>
       </c>
       <c r="E18" s="1" t="n">
@@ -881,7 +881,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Customer 17</t>
+          <t>Brightfield Logistics</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -906,17 +906,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Customer 18</t>
+          <t>Greenriver Retail</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Enterprise</t>
+          <t>SMB</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>North</t>
         </is>
       </c>
       <c r="E20" s="1" t="n">
@@ -931,7 +931,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Customer 19</t>
+          <t>Coastalpeak Foods</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -941,7 +941,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>South</t>
         </is>
       </c>
       <c r="E21" s="1" t="n">
@@ -956,17 +956,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Customer 20</t>
+          <t>Urbanpeak Logistics</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Enterprise</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>South</t>
         </is>
       </c>
       <c r="E22" s="1" t="n">
@@ -981,7 +981,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Customer 21</t>
+          <t>Brightfield Foods</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>North</t>
         </is>
       </c>
       <c r="E23" s="1" t="n">
@@ -1006,17 +1006,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Customer 22</t>
+          <t>Summitstone Foods</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Enterprise</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>North</t>
         </is>
       </c>
       <c r="E24" s="1" t="n">
@@ -1031,12 +1031,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Customer 23</t>
+          <t>Coastalriver Retail</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Enterprise</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1056,12 +1056,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Customer 24</t>
+          <t>Summitstone Labs</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>SMB</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1081,12 +1081,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Customer 25</t>
+          <t>Bluestone Traders</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Enterprise</t>
+          <t>SMB</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1106,17 +1106,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Customer 26</t>
+          <t>Urbanriver Retail</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Enterprise</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>North</t>
         </is>
       </c>
       <c r="E28" s="1" t="n">
@@ -1131,12 +1131,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Customer 27</t>
+          <t>Greenstone Labs</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Enterprise</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1156,17 +1156,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Customer 28</t>
+          <t>Silvergate Textiles</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>SMB</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>North</t>
         </is>
       </c>
       <c r="E30" s="1" t="n">
@@ -1181,17 +1181,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Customer 29</t>
+          <t>Coastalbridge Retail</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>SMB</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>South</t>
         </is>
       </c>
       <c r="E31" s="1" t="n">
@@ -1206,17 +1206,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Customer 30</t>
+          <t>Northstone Retail</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>SMB</t>
+          <t>Enterprise</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>East</t>
         </is>
       </c>
       <c r="E32" s="1" t="n">
@@ -1231,7 +1231,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Customer 31</t>
+          <t>Mapleriver Textiles</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1241,7 +1241,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>West</t>
         </is>
       </c>
       <c r="E33" s="1" t="n">
@@ -1256,17 +1256,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Customer 32</t>
+          <t>Urbanstone Foods</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>SMB</t>
+          <t>Enterprise</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>South</t>
         </is>
       </c>
       <c r="E34" s="1" t="n">
@@ -1281,7 +1281,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Customer 33</t>
+          <t>Summitgate Systems</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1306,17 +1306,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Customer 34</t>
+          <t>Bluefield Foods</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>SMB</t>
+          <t>Enterprise</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>West</t>
         </is>
       </c>
       <c r="E36" s="1" t="n">
@@ -1331,7 +1331,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Customer 35</t>
+          <t>Northriver Systems</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1341,7 +1341,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>South</t>
         </is>
       </c>
       <c r="E37" s="1" t="n">
@@ -1356,17 +1356,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Customer 36</t>
+          <t>Primeriver Studios</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Enterprise</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>West</t>
         </is>
       </c>
       <c r="E38" s="1" t="n">
@@ -1381,17 +1381,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Customer 37</t>
+          <t>Summitleaf Traders</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>SMB</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>West</t>
         </is>
       </c>
       <c r="E39" s="1" t="n">
@@ -1406,12 +1406,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Customer 38</t>
+          <t>Greenworks Retail</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>SMB</t>
+          <t>Enterprise</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1431,17 +1431,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Customer 39</t>
+          <t>Urbanfield Retail</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>SMB</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>North</t>
         </is>
       </c>
       <c r="E41" s="1" t="n">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Priya</t>
+          <t>Priya Menon</t>
         </is>
       </c>
     </row>
@@ -1505,7 +1505,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Arjun</t>
+          <t>Arjun Rao</t>
         </is>
       </c>
     </row>
@@ -1520,7 +1520,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Meera</t>
+          <t>Meera Iyer</t>
         </is>
       </c>
     </row>

</xml_diff>